<commit_message>
Enhancements to Data Simulator
</commit_message>
<xml_diff>
--- a/customer_requirements.xlsx
+++ b/customer_requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\dev\stunning-couscous\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D019C1E2-94E1-49B0-A5BF-94D6B339DDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9368ECC-1BCB-4F12-BF9B-795118EBBE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="1400" windowWidth="20350" windowHeight="14400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="560" yWindow="30" windowWidth="37930" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Requirements" sheetId="1" r:id="rId1"/>
@@ -657,7 +657,7 @@
         <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>43</v>
@@ -683,7 +683,7 @@
         <v>35</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>43</v>
@@ -761,7 +761,7 @@
         <v>35</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>32</v>
@@ -813,7 +813,7 @@
         <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>32</v>

</xml_diff>